<commit_message>
working on size data for OP, gitignore upate
</commit_message>
<xml_diff>
--- a/data/Incidental_Mortality_TCCHINOOK-25-02-Appendix-A-Catch-Detailed (1).xlsx
+++ b/data/Incidental_Mortality_TCCHINOOK-25-02-Appendix-A-Catch-Detailed (1).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Genoa/Documents/GitHub/PST_General/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7CDDC8A4-2EC6-BB45-A3AF-7704638A0569}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26F66B39-F105-9445-9732-DA7FE68CA077}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4520" yWindow="2980" windowWidth="28800" windowHeight="17120" tabRatio="862" firstSheet="1" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="3900" yWindow="1700" windowWidth="28800" windowHeight="17120" tabRatio="862" firstSheet="11" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TOC" sheetId="63" r:id="rId1"/>
@@ -39,7 +39,8 @@
     <sheet name="A23" sheetId="9" r:id="rId24"/>
     <sheet name="A24" sheetId="10" r:id="rId25"/>
     <sheet name="A25" sheetId="41" r:id="rId26"/>
-    <sheet name="Exec summ" sheetId="54" state="hidden" r:id="rId27"/>
+    <sheet name="Sheet1" sheetId="64" r:id="rId27"/>
+    <sheet name="Exec summ" sheetId="54" state="hidden" r:id="rId28"/>
   </sheets>
   <definedNames>
     <definedName name="OLE_LINK1" localSheetId="18">'A18'!$E$39</definedName>
@@ -37074,6 +37075,15 @@
 </file>
 
 <file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3BDDF7D5-B860-4241-AD54-803882453662}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1B00-000000000000}">
   <sheetPr codeName="Sheet26"/>
   <dimension ref="A1:H23"/>

</xml_diff>